<commit_message>
feat(testakten): Koeln-Akte Multi-Format-Unterordner ausbauen
emails/ auf fuenf Nachrichten erweitert (LG Koeln Pressestelle,
Rechtsabteilung Hafenstadt, Chefredaktion, Verteidigung). csv/headline_varianten.csv
um drei weitere Varianten ergaenzt. xlsx/fakten_und_quellenmatrix.xlsx um
Stellungnahmen-Synopse- und Headline-Bewertungs-Tabellenblaetter erweitert.
pdfs/ um Konkurrenzbericht, Terminuebersicht und Kontaktabzug-Uebersicht
ergaenzt.
</commit_message>
<xml_diff>
--- a/testakten/pressebericht-verdachtsberichterstattung-wirtschaftsverfahren-koeln/xlsx/fakten_und_quellenmatrix.xlsx
+++ b/testakten/pressebericht-verdachtsberichterstattung-wirtschaftsverfahren-koeln/xlsx/fakten_und_quellenmatrix.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrix" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Redaktionsschluss" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stellungnahmen_Synopse" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Headline_Bewertung" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -623,4 +625,210 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Partei</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Kernaussage</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Eingang</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Verwendung im Text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Hafenstadt Projektbau AG</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bestreitet systematische Bilanzmanipulation, verweist auf externes Gutachten</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>28.06.2026</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Zitat gekuerzt, Kern erhalten</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Verteidigung Dr. Kurth</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Verlaesslichkeit auf Fachabteilungen und Abschlusspruefer, kein persoenlicher Vorteil ersichtlich</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>03.07.2026 (Frist bis 10.07.2026)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>vollstaendige Wiedergabe vorgesehen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Staatsanwaltschaft Koeln</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Hinreichender Tatverdacht laut Pressemitteilung, keine Schuldfeststellung</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>20.06.2026</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Einordnung als Verdacht, nicht als Tatsache</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Aufsichtsrat (anonyme Quelle)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hinweis auf interne Spannungen vor Bilanzskandal</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>muendlich, 22.06.2026</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nicht namentlich verwendbar, nur als Hintergrund</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Variante</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Rechtliches Risiko</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Empfehlung</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ex-Finanzchefin vor Gericht</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>niedrig</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>verwendbar</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Millionenbetrug bei Projektbau</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>mittel</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Verdachtscharakter ergaenzen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Die Frau hinter dem Bauskandal</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>hoch</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>nicht verwenden, Vorverurteilung</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>